<commit_message>
Atualizar planilha CVM [2026-03-11]
</commit_message>
<xml_diff>
--- a/patrimonio_liquido_cvm.xlsx
+++ b/patrimonio_liquido_cvm.xlsx
@@ -415,78 +415,87 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Campo</t>
+          <t>Fundo</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Valor</t>
+          <t>CNPJ</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Competência</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Patrimônio Líquido</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Data Recebimento</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Fundo</t>
+          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
+          <t>08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>R$ 27.376.309.196,54</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>05/03/2026 14:25:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CNPJ</t>
+          <t>Nome do Fundo/Classe: ITAÚ SOBERANO RENDA FIXA SIMPLES FIF DA CIC RESPONSABILIDADE LIMITADA CNPJ: 06.175.696/0001-73</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>08.915.927/0001-63</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Competência</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+          <t>06.175.696/0001-73</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>02/2026</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Patrimônio Líquido</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>R$ 27.376.309.196,54</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Data Recebimento</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>05/03/2026 14:25:18</t>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>R$ 46.404.535.645,45</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>10/03/2026 01:34:03</t>
         </is>
       </c>
     </row>
@@ -501,16 +510,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Fundo</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>CNPJ</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Valores - Mercado</t>
         </is>
@@ -519,141 +538,361 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Disponibilidades Descrição: Disponibilidade</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="D2" t="n">
         <v>7866235.31</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Operações Compromissadas Cod. SELIC: 100000 Venc.: 01/01/2029</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="D3" t="n">
         <v>4492619539.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Operações Compromissadas Cod. SELIC: 950199 Venc.: 01/01/2029</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="D4" t="n">
         <v>2193665208.65</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>Títulos Públicos Cod. SELIC: 210100 Venc.: 01/03/2027</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="D5" t="n">
         <v>8195811298.63</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>Títulos Públicos Cod. SELIC: 210100 Venc.: 01/09/2027</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="D6" t="n">
         <v>3398933538.09</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>Títulos Públicos Cod. SELIC: 210100 Venc.: 01/03/2028</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="D7" t="n">
         <v>3067815717.22</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>Títulos Públicos Cod. SELIC: 210100 Venc.: 01/09/2028</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="D8" t="n">
         <v>2227581157.19</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>Títulos Públicos Cod. SELIC: 210100 Venc.: 01/03/2029</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="D9" t="n">
         <v>1579098012.86</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>Títulos Públicos Cod. SELIC: 210100 Venc.: 01/03/2030</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="D10" t="n">
         <v>1025819021.27</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>Títulos Públicos Cod. SELIC: 210100 Venc.: 01/09/2029</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="D11" t="n">
         <v>679121922.52</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>Títulos Públicos Cod. SELIC: 210100 Venc.: 01/09/2026</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="D12" t="n">
         <v>463364785.09</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>Títulos Públicos Cod. SELIC: 210100 Venc.: 01/03/2026</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="D13" t="n">
         <v>47767196.42</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>Valores a pagar Descrição: Valores a Pagar</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="D14" t="n">
         <v>3155171.44</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Nome do Fundo/Classe: BEM TPF FI FINANCEIRO - CI RF SIMPLES - RESP LIMITADA CNPJ: 08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>08.915.927/0001-63</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>Valores a receber Descrição: Valores a Receber</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="D15" t="n">
         <v>73523</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Nome do Fundo/Classe: ITAÚ SOBERANO RENDA FIXA SIMPLES FIF DA CIC RESPONSABILIDADE LIMITADA CNPJ: 06.175.696/0001-73</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06.175.696/0001-73</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Cotas de Fundos</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>46409482128</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Nome do Fundo/Classe: ITAÚ SOBERANO RENDA FIXA SIMPLES FIF DA CIC RESPONSABILIDADE LIMITADA CNPJ: 06.175.696/0001-73</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06.175.696/0001-73</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Disponibilidades</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>65693</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Nome do Fundo/Classe: ITAÚ SOBERANO RENDA FIXA SIMPLES FIF DA CIC RESPONSABILIDADE LIMITADA CNPJ: 06.175.696/0001-73</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06.175.696/0001-73</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Valores a pagar</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>5060751</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Nome do Fundo/Classe: ITAÚ SOBERANO RENDA FIXA SIMPLES FIF DA CIC RESPONSABILIDADE LIMITADA CNPJ: 06.175.696/0001-73</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>06.175.696/0001-73</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Valores a receber</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>48575</v>
       </c>
     </row>
   </sheetData>
@@ -667,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -690,40 +929,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Títulos Públicos</t>
+          <t>Cotas de Fundos</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20685312649.29</v>
+        <v>46409482128</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7554155888736424</v>
+        <v>0.628877357502268</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Operações Compromissadas</t>
+          <t>Títulos Públicos</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6686284748.15</v>
+        <v>20685312649.29</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2441792307438946</v>
+        <v>0.2802988562146736</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Disponibilidades</t>
+          <t>Operações Compromissadas</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7866235.31</v>
+        <v>6686284748.15</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0002872703390889405</v>
+        <v>0.09060331835479364</v>
       </c>
     </row>
     <row r="5">
@@ -733,23 +972,36 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3155171.44</v>
+        <v>8215922.439999999</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0001152250261697982</v>
+        <v>0.0001113308607766929</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Disponibilidades</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>7931928.31</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0001074825636220732</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Valores a receber</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>73523</v>
-      </c>
-      <c r="C6" t="n">
-        <v>2.685017204352634e-06</v>
+      <c r="B7" t="n">
+        <v>122098</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1.654503865924111e-06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>